<commit_message>
arrang side menu transfert multiple
</commit_message>
<xml_diff>
--- a/public/assets/fichierdeBase.xlsx
+++ b/public/assets/fichierdeBase.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP PAVILION\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{133E797E-E1E8-4B14-8BF9-9BDCC8E9265F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35231E92-F981-480A-AF6D-E0D9946F63A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AEC708BF-54C0-4D9C-B697-A0A63148652D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AEC708BF-54C0-4D9C-B697-A0A63148652D}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>prenom</t>
   </si>
@@ -48,9 +48,6 @@
     <t>typeBeneficiaire</t>
   </si>
   <si>
-    <t>numeroCompte</t>
-  </si>
-  <si>
     <t>bic</t>
   </si>
   <si>
@@ -70,6 +67,12 @@
   </si>
   <si>
     <t>objetPaiement</t>
+  </si>
+  <si>
+    <t>cleRib</t>
+  </si>
+  <si>
+    <t xml:space="preserve">numeroCompte </t>
   </si>
 </sst>
 </file>
@@ -105,8 +108,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -421,7 +427,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E99E2CD-AF32-431A-A303-F3500F268AA6}">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="15.6640625" customWidth="1"/>
@@ -430,41 +436,46 @@
     <col min="8" max="8" width="19.21875" customWidth="1"/>
     <col min="9" max="9" width="16.5546875" customWidth="1"/>
     <col min="10" max="10" width="13.88671875" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
-      </c>
-      <c r="K1" t="s">
-        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>